<commit_message>
Refresh weekly data: NNDSS 2026 + alerts 2026-05-09
</commit_message>
<xml_diff>
--- a/us/processed/state_per_disease/ウイルス性肝炎.xlsx
+++ b/us/processed/state_per_disease/ウイルス性肝炎.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q59"/>
+  <dimension ref="A1:R59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -513,6 +513,11 @@
           <t>2026-W16</t>
         </is>
       </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>2026-W17</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -568,6 +573,9 @@
       <c r="Q2" t="n">
         <v>32</v>
       </c>
+      <c r="R2" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -623,6 +631,9 @@
       <c r="Q3" t="n">
         <v>0</v>
       </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -678,6 +689,9 @@
       <c r="Q4" t="n">
         <v>0</v>
       </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -733,6 +747,9 @@
       <c r="Q5" t="n">
         <v>4</v>
       </c>
+      <c r="R5" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -788,6 +805,9 @@
       <c r="Q6" t="n">
         <v>5</v>
       </c>
+      <c r="R6" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -843,6 +863,9 @@
       <c r="Q7" t="n">
         <v>78</v>
       </c>
+      <c r="R7" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -898,6 +921,9 @@
       <c r="Q8" t="n">
         <v>125</v>
       </c>
+      <c r="R8" t="n">
+        <v>127</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -953,6 +979,9 @@
       <c r="Q9" t="n">
         <v>0</v>
       </c>
+      <c r="R9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1008,6 +1037,9 @@
       <c r="Q10" t="n">
         <v>0</v>
       </c>
+      <c r="R10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1063,6 +1095,9 @@
       <c r="Q11" t="n">
         <v>0</v>
       </c>
+      <c r="R11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1118,6 +1153,9 @@
       <c r="Q12" t="n">
         <v>0</v>
       </c>
+      <c r="R12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1173,6 +1211,9 @@
       <c r="Q13" t="n">
         <v>649</v>
       </c>
+      <c r="R13" t="n">
+        <v>692</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1228,6 +1269,9 @@
       <c r="Q14" t="n">
         <v>103</v>
       </c>
+      <c r="R14" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1283,6 +1327,9 @@
       <c r="Q15" t="n">
         <v>0</v>
       </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1338,6 +1385,9 @@
       <c r="Q16" t="n">
         <v>0</v>
       </c>
+      <c r="R16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1393,6 +1443,9 @@
       <c r="Q17" t="n">
         <v>5</v>
       </c>
+      <c r="R17" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1448,6 +1501,9 @@
       <c r="Q18" t="n">
         <v>19</v>
       </c>
+      <c r="R18" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1503,6 +1559,9 @@
       <c r="Q19" t="n">
         <v>19</v>
       </c>
+      <c r="R19" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1558,6 +1617,9 @@
       <c r="Q20" t="n">
         <v>0</v>
       </c>
+      <c r="R20" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1613,6 +1675,9 @@
       <c r="Q21" t="n">
         <v>1</v>
       </c>
+      <c r="R21" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1668,6 +1733,9 @@
       <c r="Q22" t="n">
         <v>85</v>
       </c>
+      <c r="R22" t="n">
+        <v>94</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1723,6 +1791,9 @@
       <c r="Q23" t="n">
         <v>0</v>
       </c>
+      <c r="R23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1778,6 +1849,9 @@
       <c r="Q24" t="n">
         <v>31</v>
       </c>
+      <c r="R24" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1833,6 +1907,9 @@
       <c r="Q25" t="n">
         <v>32</v>
       </c>
+      <c r="R25" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1888,6 +1965,9 @@
       <c r="Q26" t="n">
         <v>53</v>
       </c>
+      <c r="R26" t="n">
+        <v>55</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1943,6 +2023,9 @@
       <c r="Q27" t="n">
         <v>25</v>
       </c>
+      <c r="R27" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1998,6 +2081,9 @@
       <c r="Q28" t="n">
         <v>8</v>
       </c>
+      <c r="R28" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2053,6 +2139,9 @@
       <c r="Q29" t="n">
         <v>7</v>
       </c>
+      <c r="R29" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2108,6 +2197,9 @@
       <c r="Q30" t="n">
         <v>0</v>
       </c>
+      <c r="R30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2163,6 +2255,9 @@
       <c r="Q31" t="n">
         <v>7</v>
       </c>
+      <c r="R31" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2218,6 +2313,9 @@
       <c r="Q32" t="n">
         <v>2</v>
       </c>
+      <c r="R32" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -2273,6 +2371,9 @@
       <c r="Q33" t="n">
         <v>23</v>
       </c>
+      <c r="R33" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -2328,6 +2429,9 @@
       <c r="Q34" t="n">
         <v>6</v>
       </c>
+      <c r="R34" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -2383,6 +2487,9 @@
       <c r="Q35" t="n">
         <v>20</v>
       </c>
+      <c r="R35" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2438,6 +2545,9 @@
       <c r="Q36" t="n">
         <v>0</v>
       </c>
+      <c r="R36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2493,6 +2603,9 @@
       <c r="Q37" t="n">
         <v>64</v>
       </c>
+      <c r="R37" t="n">
+        <v>69</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -2548,6 +2661,9 @@
       <c r="Q38" t="n">
         <v>23</v>
       </c>
+      <c r="R38" t="n">
+        <v>23</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -2603,6 +2719,9 @@
       <c r="Q39" t="n">
         <v>33</v>
       </c>
+      <c r="R39" t="n">
+        <v>34</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -2658,6 +2777,9 @@
       <c r="Q40" t="n">
         <v>2</v>
       </c>
+      <c r="R40" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -2713,6 +2835,9 @@
       <c r="Q41" t="n">
         <v>44</v>
       </c>
+      <c r="R41" t="n">
+        <v>47</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2768,6 +2893,9 @@
       <c r="Q42" t="n">
         <v>5</v>
       </c>
+      <c r="R42" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -2823,6 +2951,9 @@
       <c r="Q43" t="n">
         <v>18</v>
       </c>
+      <c r="R43" t="n">
+        <v>21</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -2878,6 +3009,9 @@
       <c r="Q44" t="n">
         <v>40</v>
       </c>
+      <c r="R44" t="n">
+        <v>46</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -2933,6 +3067,9 @@
       <c r="Q45" t="n">
         <v>1</v>
       </c>
+      <c r="R45" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2988,6 +3125,9 @@
       <c r="Q46" t="n">
         <v>5</v>
       </c>
+      <c r="R46" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -3043,6 +3183,9 @@
       <c r="Q47" t="n">
         <v>17</v>
       </c>
+      <c r="R47" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3098,6 +3241,9 @@
       <c r="Q48" t="n">
         <v>0</v>
       </c>
+      <c r="R48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -3153,6 +3299,9 @@
       <c r="Q49" t="n">
         <v>74</v>
       </c>
+      <c r="R49" t="n">
+        <v>81</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -3208,6 +3357,9 @@
       <c r="Q50" t="n">
         <v>16</v>
       </c>
+      <c r="R50" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -3263,6 +3415,9 @@
       <c r="Q51" t="n">
         <v>1</v>
       </c>
+      <c r="R51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -3318,6 +3473,9 @@
       <c r="Q52" t="n">
         <v>0</v>
       </c>
+      <c r="R52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -3373,6 +3531,9 @@
       <c r="Q53" t="n">
         <v>27</v>
       </c>
+      <c r="R53" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -3428,6 +3589,9 @@
       <c r="Q54" t="n">
         <v>7</v>
       </c>
+      <c r="R54" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -3483,6 +3647,9 @@
       <c r="Q55" t="n">
         <v>33</v>
       </c>
+      <c r="R55" t="n">
+        <v>36</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -3538,6 +3705,9 @@
       <c r="Q56" t="n">
         <v>10</v>
       </c>
+      <c r="R56" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -3593,6 +3763,9 @@
       <c r="Q57" t="n">
         <v>25</v>
       </c>
+      <c r="R57" t="n">
+        <v>27</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -3648,6 +3821,9 @@
       <c r="Q58" t="n">
         <v>16</v>
       </c>
+      <c r="R58" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -3701,6 +3877,9 @@
         <v>0</v>
       </c>
       <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3780,7 +3959,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7">
@@ -3790,7 +3969,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>78</v>
+        <v>87</v>
       </c>
     </row>
     <row r="8">
@@ -3800,7 +3979,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9">
@@ -3850,7 +4029,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>649</v>
+        <v>692</v>
       </c>
     </row>
     <row r="14">
@@ -3890,7 +4069,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18">
@@ -3910,7 +4089,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -3930,7 +4109,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -3940,7 +4119,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="23">
@@ -3960,7 +4139,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="25">
@@ -3970,7 +4149,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="26">
@@ -3980,7 +4159,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27">
@@ -4040,7 +4219,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="33">
@@ -4050,7 +4229,7 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34">
@@ -4090,7 +4269,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="38">
@@ -4110,7 +4289,7 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="40">
@@ -4130,7 +4309,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42">
@@ -4150,7 +4329,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="44">
@@ -4160,7 +4339,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
     <row r="45">
@@ -4170,7 +4349,7 @@
         </is>
       </c>
       <c r="B45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="46">
@@ -4210,7 +4389,7 @@
         </is>
       </c>
       <c r="B49" t="n">
-        <v>74</v>
+        <v>81</v>
       </c>
     </row>
     <row r="50">
@@ -4230,7 +4409,7 @@
         </is>
       </c>
       <c r="B51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="52">
@@ -4250,7 +4429,7 @@
         </is>
       </c>
       <c r="B53" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="54">
@@ -4270,7 +4449,7 @@
         </is>
       </c>
       <c r="B55" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="56">
@@ -4280,7 +4459,7 @@
         </is>
       </c>
       <c r="B56" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57">
@@ -4290,7 +4469,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="58">
@@ -4300,7 +4479,7 @@
         </is>
       </c>
       <c r="B58" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="59">

</xml_diff>